<commit_message>
On branch master Changes to be committed: 	modified:   brick_work_calculation.xlsx
</commit_message>
<xml_diff>
--- a/other/Brick_work_calculation/brick_work_calculation.xlsx
+++ b/other/Brick_work_calculation/brick_work_calculation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Abdul\Documents\gitFiles\cheatsheets\other\Brick_work_calculation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79382414-EDDD-43C2-95A3-165AEF13C740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542F0C87-D2F1-4494-BF50-2346033DA6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,57 +34,81 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
-  <si>
-    <t>Brick_width</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Wall_width</t>
-  </si>
-  <si>
-    <t>Wall_length</t>
-  </si>
-  <si>
-    <t>Wall_height</t>
-  </si>
-  <si>
-    <t>Brick_height</t>
-  </si>
-  <si>
-    <t>Brick_lenght</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Motar (1cm)</t>
-  </si>
-  <si>
-    <t>Grand_total</t>
-  </si>
-  <si>
-    <t>Length+Motar</t>
-  </si>
-  <si>
-    <t>Height+Motar</t>
-  </si>
-  <si>
-    <t>Width+Motar</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>Devide into Fit</t>
   </si>
   <si>
-    <t>Door (3x6)</t>
-  </si>
-  <si>
-    <t>Window (4*5)</t>
-  </si>
-  <si>
-    <t>No. of Bricks without Door&amp;Window</t>
-  </si>
-  <si>
-    <t>No. of Bricks with Door&amp;Window</t>
+    <t>Length</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>Brick size (in inch)</t>
+  </si>
+  <si>
+    <t>Brick size with mortar</t>
+  </si>
+  <si>
+    <t>Mortar (cm)</t>
+  </si>
+  <si>
+    <t>WALL</t>
+  </si>
+  <si>
+    <t>BRICK</t>
+  </si>
+  <si>
+    <t>Wall size (in fit)</t>
+  </si>
+  <si>
+    <t>DOOR</t>
+  </si>
+  <si>
+    <t>Door size (in fit)</t>
+  </si>
+  <si>
+    <t>WINDOW</t>
+  </si>
+  <si>
+    <t>Window size (in fit)</t>
+  </si>
+  <si>
+    <t>Square fit</t>
+  </si>
+  <si>
+    <t>Door &amp; Window sqft</t>
+  </si>
+  <si>
+    <t>Square fit of wall after deduction</t>
+  </si>
+  <si>
+    <t>Square fit of wall</t>
+  </si>
+  <si>
+    <t>Volume of Brick</t>
+  </si>
+  <si>
+    <t>Volume of Wall</t>
+  </si>
+  <si>
+    <t>Width of Wall (in inch)</t>
+  </si>
+  <si>
+    <t>Convert into fit</t>
+  </si>
+  <si>
+    <t>Devide into inch</t>
+  </si>
+  <si>
+    <t>Number of Bricks</t>
+  </si>
+  <si>
+    <t>Volume of Wall without deduction</t>
   </si>
 </sst>
 </file>
@@ -120,10 +144,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -405,14 +435,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -420,137 +449,297 @@
     <col min="10" max="10" width="30.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>0.39300000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="3">
+        <f>SUM(B3+D8)</f>
+        <v>9.3930000000000007</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="3">
+        <f>SUM(B4+D8)</f>
+        <v>4.8929999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="3">
+        <f>SUM(B5+D8)</f>
+        <v>3.3929999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="2">
+        <f>SUM(B9*B10*B11)</f>
+        <v>155.94210695699999</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D13" s="2">
+        <f>SUM(B13/1728)</f>
+        <v>9.0244274859375001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20">
+        <f>B18*B19</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>9</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21">
+        <f>B21/12</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B26">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28">
+        <f>B26*B27</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35">
+        <f>B33*B34</f>
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>9</v>
-      </c>
-      <c r="B2">
-        <v>4.5</v>
-      </c>
-      <c r="C2">
-        <v>2.68</v>
-      </c>
-      <c r="D2">
-        <f>SUM(A2*B2*C2)</f>
-        <v>108.54</v>
-      </c>
-      <c r="E2">
-        <v>0.39400000000000002</v>
-      </c>
-      <c r="F2">
-        <f>SUM(A2+E2)</f>
-        <v>9.3940000000000001</v>
-      </c>
-      <c r="G2">
-        <f>SUM(B2+E2)</f>
-        <v>4.8940000000000001</v>
-      </c>
-      <c r="H2">
-        <f>SUM(C2+E2)</f>
-        <v>3.0740000000000003</v>
-      </c>
-      <c r="I2">
-        <f>SUM(F2*G2*H2)</f>
-        <v>141.32480146400002</v>
-      </c>
-      <c r="J2">
-        <f>SUM(I2/1728)</f>
-        <v>8.178518603240742E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" s="1" t="s">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="B37">
+        <f>B28+B35</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>0.75</v>
-      </c>
-      <c r="C5">
-        <v>10</v>
-      </c>
-      <c r="D5">
-        <f>SUM(A5*C5)</f>
-        <v>100</v>
-      </c>
-      <c r="E5">
-        <f>SUM(3*6)</f>
-        <v>18</v>
-      </c>
-      <c r="F5">
-        <f>SUM(4*5)</f>
-        <v>20</v>
-      </c>
-      <c r="G5">
-        <f>SUM(E5+F5)</f>
-        <v>38</v>
-      </c>
-      <c r="I5">
-        <f>SUM((D5*B5)/J2)</f>
-        <v>917.03649081731271</v>
+      <c r="B39" s="1">
+        <f>B20-B37</f>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>19</v>
+      </c>
+      <c r="B41">
+        <f>B39*D21</f>
+        <v>57.75</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>23</v>
+      </c>
+      <c r="B42">
+        <f>B41/D13</f>
+        <v>639.92979155730518</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44">
+        <f>B20*D21</f>
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>23</v>
+      </c>
+      <c r="B45">
+        <f>B44/D13</f>
+        <v>914.18541651043597</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>